<commit_message>
Add operation archive to source Excel report
</commit_message>
<xml_diff>
--- a/Витрати.xlsb (1).xlsx
+++ b/Витрати.xlsb (1).xlsx
@@ -15,6 +15,7 @@
   <sheets>
     <sheet name="Лист2" sheetId="2" r:id="rId1"/>
     <sheet name="Лист1" sheetId="1" r:id="rId2"/>
+    <sheet name="Останні операції" sheetId="3" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -2907,4 +2908,198 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Категорія</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Сума</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Учасник</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Коментар</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>14b35611-5463-4f15-955c-6fd5a7e24d75</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Дохід</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Інше</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>17000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Михайло</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>кукукук</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Дохід</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Зарплата</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>21400</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Михайло</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Витрата</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Продукти</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2450</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Сім’я</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Витрата</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Квартира</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>8100</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Михайло</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G5"/>
+</worksheet>
 </file>
</xml_diff>